<commit_message>
fix(upload): use image questions in tree XLSForm
</commit_message>
<xml_diff>
--- a/apps/bumicerts/public/templates/tree-data-detailed-xlsform.xlsx
+++ b/apps/bumicerts/public/templates/tree-data-detailed-xlsform.xlsx
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -582,7 +582,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Whole Tree Photo URL</t>
+          <t>Whole Tree Photo</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -602,17 +602,29 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Publicly accessible URL to a whole-tree photo; no sign-in required.</t>
-        </is>
-      </c>
-      <c r="F16"/>
-      <c r="G16"/>
-      <c r="H16"/>
+          <t>Take or choose a whole-tree photo. Export Kobo Media Attachments ZIP with your CSV.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -622,7 +634,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Leaf Photo URL</t>
+          <t>Leaf Photo</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -632,17 +644,29 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Publicly accessible URL to a leaf photo; no sign-in required.</t>
-        </is>
-      </c>
-      <c r="F17"/>
-      <c r="G17"/>
-      <c r="H17"/>
+          <t>Take or choose a leaf photo. Export Kobo Media Attachments ZIP with your CSV.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -652,7 +676,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Bark Photo URL</t>
+          <t>Bark Photo</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -662,17 +686,29 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Publicly accessible URL to a bark photo; no sign-in required.</t>
-        </is>
-      </c>
-      <c r="F18"/>
-      <c r="G18"/>
-      <c r="H18"/>
+          <t>Take or choose a bark photo. Export Kobo Media Attachments ZIP with your CSV.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -682,7 +718,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Generic Photo URL(s)</t>
+          <t>Additional Photo</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -692,12 +728,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Public photo URL(s). Separate multiple URLs with commas or semicolons.</t>
-        </is>
-      </c>
-      <c r="F19"/>
-      <c r="G19"/>
-      <c r="H19"/>
+          <t>Optional additional tree photo. Export Kobo Media Attachments ZIP with your CSV.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>